<commit_message>
melengkapi jam operasional dan layanan klinik, memperbaiki batas kecamatan
</commit_message>
<xml_diff>
--- a/data/raw/klinik_tambahan_surabaya_barat.xlsx
+++ b/data/raw/klinik_tambahan_surabaya_barat.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keterangan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Klinik_Tambahan'!$A$1:$N$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Klinik_Tambahan'!$A$1:$N$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -911,8 +911,16 @@
           <t>Dokter umum</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Mo-Sa 09:00-12:00, 17:00-21:00</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Verifikasi manual</t>
+        </is>
+      </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
           <t>Tidak lengkap; Minggu tutup</t>
@@ -965,8 +973,16 @@
           <t>Dokter gigi</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Mo-Fr 09:00-21:00; Sa 09:00-15:00</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Verifikasi manual</t>
+        </is>
+      </c>
       <c r="J8" s="3" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -1015,8 +1031,16 @@
           <t>Dokter gigi</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Mo-Fr 12:00-20:00; Sa 09:00-17:00; Su 09:00-15:00</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Verifikasi manual</t>
+        </is>
+      </c>
       <c r="J9" s="3" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
@@ -1065,8 +1089,16 @@
           <t>Dokter gigi</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Mo-Fr 08:00-22:00; Sa-Su 10:00-18:00</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Verifikasi manual</t>
+        </is>
+      </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
           <t>Senin 08.00 – 22.00 (hari lain tidak tercantum)</t>
@@ -1239,8 +1271,16 @@
           <t>Dokter gigi</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Mo 09:00-18:00; Tu-Fr 10:00-19:00; Sa 08:00-17:00, Su 08:00-16:00</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Verifikasi manual</t>
+        </is>
+      </c>
       <c r="J13" s="3" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
@@ -1518,22 +1558,22 @@
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Dokter umum</t>
+          <t>Dokter umum, Dokter gigi</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>24 jam</t>
+          <t>Mo-Su 08:00-21:00</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Lokanesia (data faskes BPJS)</t>
+          <t>Instagram resmi klinik</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Senin – Minggu 24 jam</t>
+          <t>Instagram: Poli Umum 08.00 – 21.00, Poli Gigi 19.00 – 21.00. Lokanesia (2020): Senin – Minggu 24 jam</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1551,7 +1591,11 @@
           <t>Belum dicek</t>
         </is>
       </c>
-      <c r="N18" s="3" t="inlineStr"/>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>Jam pada Instagram resmi klinik (https://www.instagram.com/klinikperdanahusada/) menggantikan data 24 jam dari Lokanesia tahun 2020. Hari operasional mengikuti Lokanesia karena Instagram tidak mencantumkan hari.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1611,8 +1655,318 @@
       </c>
       <c r="N19" s="3" t="inlineStr"/>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Praktik dr. Hendra Cipta, M.Biomed, Sp.PD (Klinik Anugerah Medika)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Citraland Gwalk Shop House W2 No. 1, Lontar</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Sambikerep</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Penyakit dalam</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Mo-Fr 18:00-22:00</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>AlamatSehat</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Senin – Jumat 18.00 – 22.00</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>https://alamatsehat.com/dokter-penyakit-dalam-di-surabaya-barat/</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>14 Agustus 2025</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>Belum dicek</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>Peta lokasi pada sumber: https://maps.app.goo.gl/EcEKdhzrnZJ1T7ye7</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Praktik dr. Iman Rachmanto, Sp.OG</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Jl. Kendung No. 61, Sememi</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Benowo</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Dokter kandungan</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Tu,Th,Fr 18:30-22:30</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Verifikasi manual</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Selasa, Kamis, dan Jumat 18.30 – 22.30 WIB</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>https://alamatsehat.com/praktek-dokter-kandungan-di-surabaya-barat/</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>11 Agustus 2025</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Terverifikasi</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>Klinik pribadi (praktik dr. Iman). Koordinat diambil dari peta lokasi pada sumber: https://maps.app.goo.gl/bkuuepkTetKn7xeQ7</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Praktik dr. Chandra Thaytty, Sp.OG</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Jl. Raya Kupang Baru No. 72, Sonokwijenan</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Sukomanunggal</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Dokter kandungan</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Mo-Sa 12:15-18:00</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Senin – Sabtu 12.15 – 18.00; Minggu dan hari besar tutup</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>https://alamatsehat.com/praktek-dokter-kandungan-di-surabaya-barat/</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>11 Agustus 2025</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>Terverifikasi</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>Jam praktik dari profil Google: https://www.google.com/searchviewer/10?svid=CAwSHRIbCgNwdnESFENnMHZaeTh4TVdNMmNuaGpZbXgzGAo. Koordinat diambil dari peta lokasi pada sumber: https://maps.app.goo.gl/28YJb6YrkJP5xYpn7</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Praktik dr. Eston A. Hadibrata, Sp.OG</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Jl. Darmo Baru Barat, Sonokwijenan</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Sukomanunggal</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="n"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Dokter kandungan</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Tu 19:00-20:30; Fr 19:15-20:30</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Waze</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Selasa 19.00 – 20.30; Jumat 19.15 – 20.30</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>https://alamatsehat.com/praktek-dokter-kandungan-di-surabaya-barat/</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>11 Agustus 2025</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>Terverifikasi</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="inlineStr">
+        <is>
+          <t>Jam praktik dari Waze: https://www.waze.com/id/live-map/directions/id/jawa-timur/dr.-eston-a-hadibrata,-sp.og?to=place.ChIJf1hp3hD81y0R0g6zUp9vXhI. Koordinat diambil dari peta lokasi pada sumber: https://maps.app.goo.gl/MhE8dakw8pkK8WCZ7</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Praktik dr. Silvya Chandra, Sp.OG (Apotek Moren Farma)</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Jl. Darmo Indah Timur Blok SS No. 19</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Tandes</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="n"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Dokter kandungan</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Mo-Sa 18:00-21:00</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Senin – Sabtu 18.00 – 21.00; Minggu dan hari libur tutup</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>https://alamatsehat.com/praktek-dokter-kandungan-di-surabaya-barat/</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>11 Agustus 2025</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>Terverifikasi</t>
+        </is>
+      </c>
+      <c r="N24" s="3" t="inlineStr">
+        <is>
+          <t>Jam praktik dari profil Google: https://www.google.com/searchviewer/10?svid=CAwSHRIbCgNwdnESFENnMHZaeTh4TVdSNGEzZzFORFZ1GAo dan https://www.google.com/searchviewer/10?svid=CAwSHRIbCgNwdnESFENnMHZaeTh4TVdadU5EVnRhM0Z6GAo. Koordinat diambil dari peta lokasi pada sumber: https://maps.app.goo.gl/GzPsnKvRG6CjrYS5A</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N19"/>
+  <autoFilter ref="A1:N24"/>
   <dataValidations count="1">
     <dataValidation sqref="M2:M218" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Belum dicek,Terverifikasi,Perlu koreksi,Tutup permanen,Tidak ditemukan"</formula1>
@@ -1628,7 +1982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1947,12 +2301,48 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
+          <t>AlamatSehat — Dokter Penyakit Dalam di Surabaya Barat</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>https://alamatsehat.com/dokter-penyakit-dalam-di-surabaya-barat/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>AlamatSehat — Praktek Dokter Kandungan di Surabaya Barat</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>https://alamatsehat.com/praktek-dokter-kandungan-di-surabaya-barat/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Waze dan profil Google</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Jam praktik dr. Eston A. Hadibrata, dr. Chandra Thaytty, dan dr. Silvya Chandra; tautan tercantum pada kolom Catatan baris terkait</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
           <t>Tanggal akses seluruh sumber</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>28 Oktober 2026</t>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>28 Oktober 2026 (sumber awal); 31 Oktober 2026 (sumber layanan spesialis)</t>
         </is>
       </c>
     </row>

</xml_diff>